<commit_message>
v3.0 - Bug fixes and project config updates
- Fix compatibility with pandas >=2.1: replace applymap with map
- Fix missing optional columns (הפסקות, הערות etc.) when source file lacks them
- Fix column order in detailed report (projects before totals)
- Add all active projects to Config: הקרן לידידות, כללי, תיכון אור, חנות, הקרן החדשה
- Add mapping: החדשה -> הקרן החדשה
- Filter empty/NaN column names from proj_cols
- Date columns display date only (no time) via datetime_format
- SUM formulas for all numeric columns including ק"מ in Total row
- Rewrite headers with bold format across all sheets

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/טבלת מיקומים.xlsx
+++ b/טבלת מיקומים.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29930"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shmuel\.gemini\antigravity\scratch\"/>
@@ -15,7 +15,7 @@
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -180,7 +180,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -580,9 +580,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB337069-6E28-4C60-8B45-BF983081CD5B}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" ht="28.5" thickBot="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -593,7 +593,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" ht="56.45" thickBot="1">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -604,7 +604,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" ht="56.45" thickBot="1">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
@@ -615,7 +615,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" ht="56.45" thickBot="1">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -626,7 +626,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" ht="56.45" thickBot="1">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -637,7 +637,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" ht="56.45" thickBot="1">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -648,7 +648,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" ht="56.45" thickBot="1">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -659,7 +659,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" ht="56.45" thickBot="1">
       <c r="A8" s="1" t="s">
         <v>4</v>
       </c>
@@ -670,7 +670,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" ht="56.45" thickBot="1">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -681,7 +681,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="42.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" ht="42.6" thickBot="1">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
@@ -692,7 +692,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" ht="56.45" thickBot="1">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
@@ -703,7 +703,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" ht="56.45" thickBot="1">
       <c r="A12" s="1" t="s">
         <v>6</v>
       </c>
@@ -714,7 +714,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" ht="56.45" thickBot="1">
       <c r="A13" s="1" t="s">
         <v>6</v>
       </c>
@@ -725,7 +725,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" ht="56.45" thickBot="1">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
@@ -736,7 +736,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" ht="56.45" thickBot="1">
       <c r="A15" s="1" t="s">
         <v>8</v>
       </c>
@@ -747,7 +747,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="56.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" ht="56.45" thickBot="1">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>

</xml_diff>